<commit_message>
Mise à jour des profils FHIR suite issues NRISS b312ff97b92dc5cea6799cab72c96a1aa9bd0d3b
</commit_message>
<xml_diff>
--- a/issuesNRISS/ig/StructureDefinition-fr-imaging-study-document.xlsx
+++ b/issuesNRISS/ig/StructureDefinition-fr-imaging-study-document.xlsx
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-06-17T08:17:10+00:00</t>
+    <t>2026-06-18T14:12:01+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -797,7 +797,7 @@
 </t>
   </si>
   <si>
-    <t>Number of Study Related Series</t>
+    <t>Nombre de séries</t>
   </si>
   <si>
     <t>Number of Series in the Study. This value given may be larger than the number of series elements this Resource contains due to resource availability, security, or other factors. This element should be present if any series elements are present.</t>
@@ -4384,7 +4384,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="23" hidden="true">
+    <row r="23">
       <c r="A23" t="s" s="2">
         <v>245</v>
       </c>
@@ -4403,7 +4403,7 @@
         <v>89</v>
       </c>
       <c r="H23" t="s" s="2">
-        <v>78</v>
+        <v>90</v>
       </c>
       <c r="I23" t="s" s="2">
         <v>78</v>

</xml_diff>